<commit_message>
Bo goi tien trinh ngoai (PowerShell/certutil) - bi Kaspersky chan
- ClsUpdate: thay file trong zip bang Shell.Application, co gioi han cho
  va doi chieu kich thuoc sau khi chep
- ModDist: bo certutil, kiem tra file tai ve bang chu ky dinh dang + kich thuoc
- ModRibbon: doc danh sach icon tu sheet MAP thay vi giai nen customUI
- manifest: them cot kich thuoc file

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MauBieu.xlsx
+++ b/MauBieu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\00_CLAUDE\TT99_Thuong Mai\_Update_2026-08-30\gpacc-dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED8157F2-851D-44BC-8D1E-D996AF2849F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C10FF47D-1086-44A6-8B95-6B53880E871E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{E071E4E7-1758-4045-87D0-0BF1BC03A9AC}"/>
+    <workbookView xWindow="810" yWindow="1640" windowWidth="21130" windowHeight="18320" xr2:uid="{61185216-AEBC-43BB-B83F-050DAA1B6097}"/>
   </bookViews>
   <sheets>
     <sheet name="MAP" sheetId="1" r:id="rId1"/>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1415" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1810" uniqueCount="569">
   <si>
     <t>MauSo</t>
   </si>
@@ -243,7 +243,7 @@
     <t>ct23a</t>
   </si>
   <si>
-    <t>MOI - truoc day khong xuat, kiem tra truoc khi dung</t>
+    <t>DA XAC NHAN xuat (2026-08-31) - hang hoa nhap khau</t>
   </si>
   <si>
     <t>24a</t>
@@ -1390,6 +1390,420 @@
   </si>
   <si>
     <t>D34</t>
+  </si>
+  <si>
+    <t>RIBBON</t>
+  </si>
+  <si>
+    <t>ICON</t>
+  </si>
+  <si>
+    <t>TTDN</t>
+  </si>
+  <si>
+    <t>BlogHomePage</t>
+  </si>
+  <si>
+    <t>danh sach icon Ribbon - PhatHanh.ps1 sinh ra</t>
+  </si>
+  <si>
+    <t>LuuY</t>
+  </si>
+  <si>
+    <t>CommentInsert</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu1</t>
+  </si>
+  <si>
+    <t>ControlsGallery</t>
+  </si>
+  <si>
+    <t>CmdKPG</t>
+  </si>
+  <si>
+    <t>Undo</t>
+  </si>
+  <si>
+    <t>Bnt_NewFile</t>
+  </si>
+  <si>
+    <t>FileNew</t>
+  </si>
+  <si>
+    <t>ModLTinh.DownLog</t>
+  </si>
+  <si>
+    <t>ImportTextFile</t>
+  </si>
+  <si>
+    <t>ModLTinh.DownExHDSD</t>
+  </si>
+  <si>
+    <t>Help</t>
+  </si>
+  <si>
+    <t>CapNhatMauBieu</t>
+  </si>
+  <si>
+    <t>RefreshAll</t>
+  </si>
+  <si>
+    <t>KiemTraToanBoMap</t>
+  </si>
+  <si>
+    <t>FindDialog</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu2</t>
+  </si>
+  <si>
+    <t>NewAlert</t>
+  </si>
+  <si>
+    <t>customButton4</t>
+  </si>
+  <si>
+    <t>MicrosoftExcel</t>
+  </si>
+  <si>
+    <t>customButton5</t>
+  </si>
+  <si>
+    <t>ContactPictureMenu</t>
+  </si>
+  <si>
+    <t>customButton6</t>
+  </si>
+  <si>
+    <t>AddressBook</t>
+  </si>
+  <si>
+    <t>BntEmail</t>
+  </si>
+  <si>
+    <t>MicrosoftOutlook</t>
+  </si>
+  <si>
+    <t>AnSheet</t>
+  </si>
+  <si>
+    <t>Lock</t>
+  </si>
+  <si>
+    <t>NK_HDXML</t>
+  </si>
+  <si>
+    <t>AutoSummarize</t>
+  </si>
+  <si>
+    <t>BR</t>
+  </si>
+  <si>
+    <t>TableInsert</t>
+  </si>
+  <si>
+    <t>NK_Ban</t>
+  </si>
+  <si>
+    <t>AdpDiagramArrangeSelection</t>
+  </si>
+  <si>
+    <t>MV</t>
+  </si>
+  <si>
+    <t>PivotTableInsert</t>
+  </si>
+  <si>
+    <t>NK_Mua</t>
+  </si>
+  <si>
+    <t>AccessListAssets</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>SymbolInsert</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu3</t>
+  </si>
+  <si>
+    <t>SDDK_CN</t>
+  </si>
+  <si>
+    <t>GroupListNew</t>
+  </si>
+  <si>
+    <t>CN_TH</t>
+  </si>
+  <si>
+    <t>CN_CTiet</t>
+  </si>
+  <si>
+    <t>PBKH</t>
+  </si>
+  <si>
+    <t>Bang_PBo</t>
+  </si>
+  <si>
+    <t>GroupListEdit</t>
+  </si>
+  <si>
+    <t>Bang_TSCD</t>
+  </si>
+  <si>
+    <t>GroupListSummaryNew</t>
+  </si>
+  <si>
+    <t>customButton7</t>
+  </si>
+  <si>
+    <t>DateAndTimeInsert</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu6</t>
+  </si>
+  <si>
+    <t>AccessListCustomDatasheet</t>
+  </si>
+  <si>
+    <t>DK_HHDV</t>
+  </si>
+  <si>
+    <t>NXT</t>
+  </si>
+  <si>
+    <t>Subtotal</t>
+  </si>
+  <si>
+    <t>GV</t>
+  </si>
+  <si>
+    <t>AsianLayoutCharactersEnclose</t>
+  </si>
+  <si>
+    <t>BangLuong</t>
+  </si>
+  <si>
+    <t>TinhLuong</t>
+  </si>
+  <si>
+    <t>CalculateNow</t>
+  </si>
+  <si>
+    <t>CDSPS</t>
+  </si>
+  <si>
+    <t>StarRatedFull</t>
+  </si>
+  <si>
+    <t>CDSPS_NT</t>
+  </si>
+  <si>
+    <t>StarRatedEmpty</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu8</t>
+  </si>
+  <si>
+    <t>CreateReport</t>
+  </si>
+  <si>
+    <t>NKC</t>
+  </si>
+  <si>
+    <t>HTTK</t>
+  </si>
+  <si>
+    <t>GroupOutline</t>
+  </si>
+  <si>
+    <t>Giai_Trinh</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu9</t>
+  </si>
+  <si>
+    <t>WatchWindow</t>
+  </si>
+  <si>
+    <t>SDHD</t>
+  </si>
+  <si>
+    <t>SignatureShow</t>
+  </si>
+  <si>
+    <t>customButton8</t>
+  </si>
+  <si>
+    <t>Organizer</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu10</t>
+  </si>
+  <si>
+    <t>ReadingMode</t>
+  </si>
+  <si>
+    <t>AdpDiagramShowRelationshipLabels</t>
+  </si>
+  <si>
+    <t>GDLK</t>
+  </si>
+  <si>
+    <t>TabOrder</t>
+  </si>
+  <si>
+    <t>PHU_LUC_01</t>
+  </si>
+  <si>
+    <t>MoveDownCustomAction</t>
+  </si>
+  <si>
+    <t>MyDropdown_TNCN</t>
+  </si>
+  <si>
+    <t>AddOrRemoveAttendees</t>
+  </si>
+  <si>
+    <t>customButton39</t>
+  </si>
+  <si>
+    <t>PL_051</t>
+  </si>
+  <si>
+    <t>GroupInsertBarcode</t>
+  </si>
+  <si>
+    <t>PL_052</t>
+  </si>
+  <si>
+    <t>GroupInkPens</t>
+  </si>
+  <si>
+    <t>customButton42</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu12</t>
+  </si>
+  <si>
+    <t>MenuPublish</t>
+  </si>
+  <si>
+    <t>KQKD</t>
+  </si>
+  <si>
+    <t>ChartInsert</t>
+  </si>
+  <si>
+    <t>CDKT</t>
+  </si>
+  <si>
+    <t>LCTT</t>
+  </si>
+  <si>
+    <t>EquationMatrixGallery</t>
+  </si>
+  <si>
+    <t>LCGT</t>
+  </si>
+  <si>
+    <t>FormulaMoreFunctionsMenu</t>
+  </si>
+  <si>
+    <t>TMinh</t>
+  </si>
+  <si>
+    <t>AccessRelinkLists</t>
+  </si>
+  <si>
+    <t>BiaBCTC</t>
+  </si>
+  <si>
+    <t>PictureInsertFromFile</t>
+  </si>
+  <si>
+    <t>customButton11</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu13</t>
+  </si>
+  <si>
+    <t>MultiplePages</t>
+  </si>
+  <si>
+    <t>Tinh_Hinh</t>
+  </si>
+  <si>
+    <t>MailSelectNames</t>
+  </si>
+  <si>
+    <t>Tinh_Hinh1</t>
+  </si>
+  <si>
+    <t>AddInsMenu</t>
+  </si>
+  <si>
+    <t>DT_CP</t>
+  </si>
+  <si>
+    <t>TH_DKhoan</t>
+  </si>
+  <si>
+    <t>Phieu_NX</t>
+  </si>
+  <si>
+    <t>HeaderFooterInsert</t>
+  </si>
+  <si>
+    <t>MyDropdownMenu14</t>
+  </si>
+  <si>
+    <t>Bia</t>
+  </si>
+  <si>
+    <t>So_Cai</t>
+  </si>
+  <si>
+    <t>FilePrepareMenu</t>
+  </si>
+  <si>
+    <t>So_Chi_Tiet</t>
+  </si>
+  <si>
+    <t>FullPageView</t>
+  </si>
+  <si>
+    <t>So_CPKD</t>
+  </si>
+  <si>
+    <t>BuildingBlocksOrganizer</t>
+  </si>
+  <si>
+    <t>So_Quy</t>
+  </si>
+  <si>
+    <t>CalculateSheet</t>
+  </si>
+  <si>
+    <t>So_TGNH</t>
+  </si>
+  <si>
+    <t>AccountMenu</t>
+  </si>
+  <si>
+    <t>So_NKBan</t>
+  </si>
+  <si>
+    <t>So_NKMua</t>
+  </si>
+  <si>
+    <t>So_Kho</t>
+  </si>
+  <si>
+    <t>ExchangeFolder</t>
   </si>
 </sst>
 </file>
@@ -39144,9 +39558,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6651BB38-7572-41FA-885E-DBFACE864C4E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8C71918-3663-46ED-B091-3A7FBD33E275}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N160"/>
+  <dimension ref="A1:N239"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.6328125" bestFit="1" customWidth="1"/>
@@ -39156,11 +39570,11 @@
     <col min="5" max="5" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="44.6328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="30.90625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="47.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="47.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -44206,6 +44620,1349 @@
       </c>
       <c r="L160" t="s">
         <v>390</v>
+      </c>
+    </row>
+    <row r="161" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>431</v>
+      </c>
+      <c r="G161" t="s">
+        <v>432</v>
+      </c>
+      <c r="H161" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="I161" t="s">
+        <v>434</v>
+      </c>
+      <c r="L161" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="162" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>431</v>
+      </c>
+      <c r="G162" t="s">
+        <v>432</v>
+      </c>
+      <c r="H162" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="I162" t="s">
+        <v>437</v>
+      </c>
+      <c r="L162" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>431</v>
+      </c>
+      <c r="G163" t="s">
+        <v>432</v>
+      </c>
+      <c r="H163" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="I163" t="s">
+        <v>439</v>
+      </c>
+      <c r="L163" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="164" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>431</v>
+      </c>
+      <c r="G164" t="s">
+        <v>432</v>
+      </c>
+      <c r="H164" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="I164" t="s">
+        <v>441</v>
+      </c>
+      <c r="L164" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="165" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>431</v>
+      </c>
+      <c r="G165" t="s">
+        <v>432</v>
+      </c>
+      <c r="H165" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="I165" t="s">
+        <v>443</v>
+      </c>
+      <c r="L165" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="166" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>431</v>
+      </c>
+      <c r="G166" t="s">
+        <v>432</v>
+      </c>
+      <c r="H166" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="I166" t="s">
+        <v>445</v>
+      </c>
+      <c r="L166" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="167" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>431</v>
+      </c>
+      <c r="G167" t="s">
+        <v>432</v>
+      </c>
+      <c r="H167" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="I167" t="s">
+        <v>447</v>
+      </c>
+      <c r="L167" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>431</v>
+      </c>
+      <c r="G168" t="s">
+        <v>432</v>
+      </c>
+      <c r="H168" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="I168" t="s">
+        <v>449</v>
+      </c>
+      <c r="L168" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="169" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>431</v>
+      </c>
+      <c r="G169" t="s">
+        <v>432</v>
+      </c>
+      <c r="H169" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="I169" t="s">
+        <v>451</v>
+      </c>
+      <c r="L169" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="170" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>431</v>
+      </c>
+      <c r="G170" t="s">
+        <v>432</v>
+      </c>
+      <c r="H170" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="I170" t="s">
+        <v>453</v>
+      </c>
+      <c r="L170" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="171" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>431</v>
+      </c>
+      <c r="G171" t="s">
+        <v>432</v>
+      </c>
+      <c r="H171" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="I171" t="s">
+        <v>455</v>
+      </c>
+      <c r="L171" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="172" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>431</v>
+      </c>
+      <c r="G172" t="s">
+        <v>432</v>
+      </c>
+      <c r="H172" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="I172" t="s">
+        <v>457</v>
+      </c>
+      <c r="L172" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="173" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>431</v>
+      </c>
+      <c r="G173" t="s">
+        <v>432</v>
+      </c>
+      <c r="H173" s="4" t="s">
+        <v>458</v>
+      </c>
+      <c r="I173" t="s">
+        <v>459</v>
+      </c>
+      <c r="L173" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="174" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>431</v>
+      </c>
+      <c r="G174" t="s">
+        <v>432</v>
+      </c>
+      <c r="H174" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="I174" t="s">
+        <v>461</v>
+      </c>
+      <c r="L174" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="175" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>431</v>
+      </c>
+      <c r="G175" t="s">
+        <v>432</v>
+      </c>
+      <c r="H175" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="I175" t="s">
+        <v>463</v>
+      </c>
+      <c r="L175" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="176" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>431</v>
+      </c>
+      <c r="G176" t="s">
+        <v>432</v>
+      </c>
+      <c r="H176" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="I176" t="s">
+        <v>465</v>
+      </c>
+      <c r="L176" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="177" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>431</v>
+      </c>
+      <c r="G177" t="s">
+        <v>432</v>
+      </c>
+      <c r="H177" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="I177" t="s">
+        <v>467</v>
+      </c>
+      <c r="L177" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="178" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>431</v>
+      </c>
+      <c r="G178" t="s">
+        <v>432</v>
+      </c>
+      <c r="H178" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="I178" t="s">
+        <v>469</v>
+      </c>
+      <c r="L178" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="179" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>431</v>
+      </c>
+      <c r="G179" t="s">
+        <v>432</v>
+      </c>
+      <c r="H179" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="I179" t="s">
+        <v>471</v>
+      </c>
+      <c r="L179" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="180" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>431</v>
+      </c>
+      <c r="G180" t="s">
+        <v>432</v>
+      </c>
+      <c r="H180" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="I180" t="s">
+        <v>473</v>
+      </c>
+      <c r="L180" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="181" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>431</v>
+      </c>
+      <c r="G181" t="s">
+        <v>432</v>
+      </c>
+      <c r="H181" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="I181" t="s">
+        <v>475</v>
+      </c>
+      <c r="L181" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="182" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>431</v>
+      </c>
+      <c r="G182" t="s">
+        <v>432</v>
+      </c>
+      <c r="H182" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="I182" t="s">
+        <v>459</v>
+      </c>
+      <c r="L182" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>431</v>
+      </c>
+      <c r="G183" t="s">
+        <v>432</v>
+      </c>
+      <c r="H183" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="I183" t="s">
+        <v>478</v>
+      </c>
+      <c r="L183" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="184" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>431</v>
+      </c>
+      <c r="G184" t="s">
+        <v>432</v>
+      </c>
+      <c r="H184" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="I184" t="s">
+        <v>471</v>
+      </c>
+      <c r="L184" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="185" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>431</v>
+      </c>
+      <c r="G185" t="s">
+        <v>432</v>
+      </c>
+      <c r="H185" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="I185" t="s">
+        <v>467</v>
+      </c>
+      <c r="L185" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="186" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>431</v>
+      </c>
+      <c r="G186" t="s">
+        <v>432</v>
+      </c>
+      <c r="H186" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="I186" t="s">
+        <v>471</v>
+      </c>
+      <c r="L186" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="187" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>431</v>
+      </c>
+      <c r="G187" t="s">
+        <v>432</v>
+      </c>
+      <c r="H187" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="I187" t="s">
+        <v>483</v>
+      </c>
+      <c r="L187" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="188" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>431</v>
+      </c>
+      <c r="G188" t="s">
+        <v>432</v>
+      </c>
+      <c r="H188" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="I188" t="s">
+        <v>485</v>
+      </c>
+      <c r="L188" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="189" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>431</v>
+      </c>
+      <c r="G189" t="s">
+        <v>432</v>
+      </c>
+      <c r="H189" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="I189" t="s">
+        <v>487</v>
+      </c>
+      <c r="L189" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="190" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>431</v>
+      </c>
+      <c r="G190" t="s">
+        <v>432</v>
+      </c>
+      <c r="H190" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="I190" t="s">
+        <v>489</v>
+      </c>
+      <c r="L190" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="191" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>431</v>
+      </c>
+      <c r="G191" t="s">
+        <v>432</v>
+      </c>
+      <c r="H191" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I191" t="s">
+        <v>478</v>
+      </c>
+      <c r="L191" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="192" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>431</v>
+      </c>
+      <c r="G192" t="s">
+        <v>432</v>
+      </c>
+      <c r="H192" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I192" t="s">
+        <v>492</v>
+      </c>
+      <c r="L192" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="193" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>431</v>
+      </c>
+      <c r="G193" t="s">
+        <v>432</v>
+      </c>
+      <c r="H193" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="I193" t="s">
+        <v>494</v>
+      </c>
+      <c r="L193" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="194" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>431</v>
+      </c>
+      <c r="G194" t="s">
+        <v>432</v>
+      </c>
+      <c r="H194" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="I194" t="s">
+        <v>467</v>
+      </c>
+      <c r="L194" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="195" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>431</v>
+      </c>
+      <c r="G195" t="s">
+        <v>432</v>
+      </c>
+      <c r="H195" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="I195" t="s">
+        <v>497</v>
+      </c>
+      <c r="L195" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="196" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>431</v>
+      </c>
+      <c r="G196" t="s">
+        <v>432</v>
+      </c>
+      <c r="H196" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="I196" t="s">
+        <v>499</v>
+      </c>
+      <c r="L196" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="197" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>431</v>
+      </c>
+      <c r="G197" t="s">
+        <v>432</v>
+      </c>
+      <c r="H197" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="I197" t="s">
+        <v>501</v>
+      </c>
+      <c r="L197" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="198" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>431</v>
+      </c>
+      <c r="G198" t="s">
+        <v>432</v>
+      </c>
+      <c r="H198" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="I198" t="s">
+        <v>503</v>
+      </c>
+      <c r="L198" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="199" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>431</v>
+      </c>
+      <c r="G199" t="s">
+        <v>432</v>
+      </c>
+      <c r="H199" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="I199" t="s">
+        <v>465</v>
+      </c>
+      <c r="L199" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="200" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>431</v>
+      </c>
+      <c r="G200" t="s">
+        <v>432</v>
+      </c>
+      <c r="H200" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="I200" t="s">
+        <v>506</v>
+      </c>
+      <c r="L200" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="201" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>431</v>
+      </c>
+      <c r="G201" t="s">
+        <v>432</v>
+      </c>
+      <c r="H201" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="I201" t="s">
+        <v>451</v>
+      </c>
+      <c r="L201" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="202" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>431</v>
+      </c>
+      <c r="G202" t="s">
+        <v>432</v>
+      </c>
+      <c r="H202" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="I202" t="s">
+        <v>509</v>
+      </c>
+      <c r="L202" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="203" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>431</v>
+      </c>
+      <c r="G203" t="s">
+        <v>432</v>
+      </c>
+      <c r="H203" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I203" t="s">
+        <v>467</v>
+      </c>
+      <c r="L203" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="204" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>431</v>
+      </c>
+      <c r="G204" t="s">
+        <v>432</v>
+      </c>
+      <c r="H204" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="I204" t="s">
+        <v>511</v>
+      </c>
+      <c r="L204" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="205" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>431</v>
+      </c>
+      <c r="G205" t="s">
+        <v>432</v>
+      </c>
+      <c r="H205" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="I205" t="s">
+        <v>513</v>
+      </c>
+      <c r="L205" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="206" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>431</v>
+      </c>
+      <c r="G206" t="s">
+        <v>432</v>
+      </c>
+      <c r="H206" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="I206" t="s">
+        <v>515</v>
+      </c>
+      <c r="L206" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="207" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>431</v>
+      </c>
+      <c r="G207" t="s">
+        <v>432</v>
+      </c>
+      <c r="H207" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="I207" t="s">
+        <v>467</v>
+      </c>
+      <c r="L207" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="208" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>431</v>
+      </c>
+      <c r="G208" t="s">
+        <v>432</v>
+      </c>
+      <c r="H208" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="I208" t="s">
+        <v>516</v>
+      </c>
+      <c r="L208" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="209" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>431</v>
+      </c>
+      <c r="G209" t="s">
+        <v>432</v>
+      </c>
+      <c r="H209" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="I209" t="s">
+        <v>518</v>
+      </c>
+      <c r="L209" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="210" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>431</v>
+      </c>
+      <c r="G210" t="s">
+        <v>432</v>
+      </c>
+      <c r="H210" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="I210" t="s">
+        <v>520</v>
+      </c>
+      <c r="L210" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="211" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>431</v>
+      </c>
+      <c r="G211" t="s">
+        <v>432</v>
+      </c>
+      <c r="H211" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="I211" t="s">
+        <v>522</v>
+      </c>
+      <c r="L211" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="212" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
+        <v>431</v>
+      </c>
+      <c r="G212" t="s">
+        <v>432</v>
+      </c>
+      <c r="H212" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="I212" t="s">
+        <v>467</v>
+      </c>
+      <c r="L212" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="213" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A213" t="s">
+        <v>431</v>
+      </c>
+      <c r="G213" t="s">
+        <v>432</v>
+      </c>
+      <c r="H213" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="I213" t="s">
+        <v>525</v>
+      </c>
+      <c r="L213" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="214" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A214" t="s">
+        <v>431</v>
+      </c>
+      <c r="G214" t="s">
+        <v>432</v>
+      </c>
+      <c r="H214" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="I214" t="s">
+        <v>527</v>
+      </c>
+      <c r="L214" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="215" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A215" t="s">
+        <v>431</v>
+      </c>
+      <c r="G215" t="s">
+        <v>432</v>
+      </c>
+      <c r="H215" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="I215" t="s">
+        <v>465</v>
+      </c>
+      <c r="L215" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A216" t="s">
+        <v>431</v>
+      </c>
+      <c r="G216" t="s">
+        <v>432</v>
+      </c>
+      <c r="H216" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="I216" t="s">
+        <v>530</v>
+      </c>
+      <c r="L216" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A217" t="s">
+        <v>431</v>
+      </c>
+      <c r="G217" t="s">
+        <v>432</v>
+      </c>
+      <c r="H217" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="I217" t="s">
+        <v>532</v>
+      </c>
+      <c r="L217" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="218" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A218" t="s">
+        <v>431</v>
+      </c>
+      <c r="G218" t="s">
+        <v>432</v>
+      </c>
+      <c r="H218" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="I218" t="s">
+        <v>499</v>
+      </c>
+      <c r="L218" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="219" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A219" t="s">
+        <v>431</v>
+      </c>
+      <c r="G219" t="s">
+        <v>432</v>
+      </c>
+      <c r="H219" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="I219" t="s">
+        <v>535</v>
+      </c>
+      <c r="L219" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="220" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A220" t="s">
+        <v>431</v>
+      </c>
+      <c r="G220" t="s">
+        <v>432</v>
+      </c>
+      <c r="H220" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="I220" t="s">
+        <v>537</v>
+      </c>
+      <c r="L220" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="221" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A221" t="s">
+        <v>431</v>
+      </c>
+      <c r="G221" t="s">
+        <v>432</v>
+      </c>
+      <c r="H221" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="I221" t="s">
+        <v>539</v>
+      </c>
+      <c r="L221" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="222" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A222" t="s">
+        <v>431</v>
+      </c>
+      <c r="G222" t="s">
+        <v>432</v>
+      </c>
+      <c r="H222" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="I222" t="s">
+        <v>541</v>
+      </c>
+      <c r="L222" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="223" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A223" t="s">
+        <v>431</v>
+      </c>
+      <c r="G223" t="s">
+        <v>432</v>
+      </c>
+      <c r="H223" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="I223" t="s">
+        <v>513</v>
+      </c>
+      <c r="L223" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="224" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>431</v>
+      </c>
+      <c r="G224" t="s">
+        <v>432</v>
+      </c>
+      <c r="H224" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="I224" t="s">
+        <v>544</v>
+      </c>
+      <c r="L224" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="225" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>431</v>
+      </c>
+      <c r="G225" t="s">
+        <v>432</v>
+      </c>
+      <c r="H225" s="4" t="s">
+        <v>545</v>
+      </c>
+      <c r="I225" t="s">
+        <v>546</v>
+      </c>
+      <c r="L225" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="226" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>431</v>
+      </c>
+      <c r="G226" t="s">
+        <v>432</v>
+      </c>
+      <c r="H226" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="I226" t="s">
+        <v>548</v>
+      </c>
+      <c r="L226" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="227" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>431</v>
+      </c>
+      <c r="G227" t="s">
+        <v>432</v>
+      </c>
+      <c r="H227" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="I227" t="s">
+        <v>532</v>
+      </c>
+      <c r="L227" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="228" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>431</v>
+      </c>
+      <c r="G228" t="s">
+        <v>432</v>
+      </c>
+      <c r="H228" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="I228" t="s">
+        <v>492</v>
+      </c>
+      <c r="L228" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="229" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>431</v>
+      </c>
+      <c r="G229" t="s">
+        <v>432</v>
+      </c>
+      <c r="H229" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="I229" t="s">
+        <v>552</v>
+      </c>
+      <c r="L229" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="230" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>431</v>
+      </c>
+      <c r="G230" t="s">
+        <v>432</v>
+      </c>
+      <c r="H230" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="I230" t="s">
+        <v>503</v>
+      </c>
+      <c r="L230" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="231" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>431</v>
+      </c>
+      <c r="G231" t="s">
+        <v>432</v>
+      </c>
+      <c r="H231" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="I231" t="s">
+        <v>541</v>
+      </c>
+      <c r="L231" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="232" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>431</v>
+      </c>
+      <c r="G232" t="s">
+        <v>432</v>
+      </c>
+      <c r="H232" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="I232" t="s">
+        <v>556</v>
+      </c>
+      <c r="L232" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="233" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>431</v>
+      </c>
+      <c r="G233" t="s">
+        <v>432</v>
+      </c>
+      <c r="H233" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="I233" t="s">
+        <v>558</v>
+      </c>
+      <c r="L233" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="234" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>431</v>
+      </c>
+      <c r="G234" t="s">
+        <v>432</v>
+      </c>
+      <c r="H234" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="I234" t="s">
+        <v>560</v>
+      </c>
+      <c r="L234" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="235" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>431</v>
+      </c>
+      <c r="G235" t="s">
+        <v>432</v>
+      </c>
+      <c r="H235" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="I235" t="s">
+        <v>562</v>
+      </c>
+      <c r="L235" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="236" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>431</v>
+      </c>
+      <c r="G236" t="s">
+        <v>432</v>
+      </c>
+      <c r="H236" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="I236" t="s">
+        <v>564</v>
+      </c>
+      <c r="L236" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="237" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>431</v>
+      </c>
+      <c r="G237" t="s">
+        <v>432</v>
+      </c>
+      <c r="H237" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="I237" t="s">
+        <v>469</v>
+      </c>
+      <c r="L237" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="238" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>431</v>
+      </c>
+      <c r="G238" t="s">
+        <v>432</v>
+      </c>
+      <c r="H238" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="I238" t="s">
+        <v>473</v>
+      </c>
+      <c r="L238" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="239" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>431</v>
+      </c>
+      <c r="G239" t="s">
+        <v>432</v>
+      </c>
+      <c r="H239" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="I239" t="s">
+        <v>568</v>
+      </c>
+      <c r="L239" t="s">
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
phat hanh 26093001: thuyet minh BCTC tu lay so TSCD + von chu so huu nam truoc (bang va VA_BOCUC, schema 6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MauBieu.xlsx
+++ b/MauBieu.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B926AE91-A64B-452C-B1B4-E271545D7B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\00_CLAUDE\TT99_Thuong Mai\_Update_2026-08-30\gpacc-dist\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41C5156-1759-4A47-A840-0D648D3978FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{65DAC49F-DB37-4ACF-9950-1AF1DBA8E511}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="28800" windowHeight="15370" xr2:uid="{65DAC49F-DB37-4ACF-9950-1AF1DBA8E511}"/>
   </bookViews>
   <sheets>
     <sheet name="VA_BOCUC" sheetId="4" r:id="rId1"/>
@@ -74,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="227">
   <si>
     <t>NK_Mua</t>
   </si>
@@ -486,6 +491,276 @@
   <si>
     <t>=IFERROR(I28/I15,"")</t>
   </si>
+  <si>
+    <t>VA26093001_01</t>
+  </si>
+  <si>
+    <t>TMinh</t>
+  </si>
+  <si>
+    <t>M214</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(M210,Bang_CDSPS,5,0)</t>
+  </si>
+  <si>
+    <t>TM muc 9: TSCD huu hinh mua trong nam = PS No TK 211x</t>
+  </si>
+  <si>
+    <t>VA26093001_02</t>
+  </si>
+  <si>
+    <t>Q214</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(Q210,Bang_CDSPS,5,0)</t>
+  </si>
+  <si>
+    <t>VA26093001_03</t>
+  </si>
+  <si>
+    <t>U214</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(U210,Bang_CDSPS,5,0)</t>
+  </si>
+  <si>
+    <t>VA26093001_04</t>
+  </si>
+  <si>
+    <t>Y214</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(Y210,Bang_CDSPS,5,0)</t>
+  </si>
+  <si>
+    <t>VA26093001_05</t>
+  </si>
+  <si>
+    <t>AC214</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(AC210,Bang_CDSPS,5,0)</t>
+  </si>
+  <si>
+    <t>VA26093001_06</t>
+  </si>
+  <si>
+    <t>M222</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,M210,Bang_TSCD!$R$16:$R$5000)</t>
+  </si>
+  <si>
+    <t>TM muc 9: hao mon luy ke dau nam lay tu Bang_TSCD</t>
+  </si>
+  <si>
+    <t>VA26093001_07</t>
+  </si>
+  <si>
+    <t>Q222</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,Q210,Bang_TSCD!$R$16:$R$5000)</t>
+  </si>
+  <si>
+    <t>VA26093001_08</t>
+  </si>
+  <si>
+    <t>U222</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,U210,Bang_TSCD!$R$16:$R$5000)</t>
+  </si>
+  <si>
+    <t>VA26093001_09</t>
+  </si>
+  <si>
+    <t>Y222</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,Y210,Bang_TSCD!$R$16:$R$5000)</t>
+  </si>
+  <si>
+    <t>VA26093001_10</t>
+  </si>
+  <si>
+    <t>AC222</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,AC210,Bang_TSCD!$R$16:$R$5000)</t>
+  </si>
+  <si>
+    <t>VA26093001_11</t>
+  </si>
+  <si>
+    <t>M223</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,M210,Bang_TSCD!$S$16:$S$5000)</t>
+  </si>
+  <si>
+    <t>TM muc 9: khau hao trong nam lay tu Bang_TSCD</t>
+  </si>
+  <si>
+    <t>VA26093001_12</t>
+  </si>
+  <si>
+    <t>Q223</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,Q210,Bang_TSCD!$S$16:$S$5000)</t>
+  </si>
+  <si>
+    <t>VA26093001_13</t>
+  </si>
+  <si>
+    <t>U223</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,U210,Bang_TSCD!$S$16:$S$5000)</t>
+  </si>
+  <si>
+    <t>VA26093001_14</t>
+  </si>
+  <si>
+    <t>Y223</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,Y210,Bang_TSCD!$S$16:$S$5000)</t>
+  </si>
+  <si>
+    <t>VA26093001_15</t>
+  </si>
+  <si>
+    <t>AC223</t>
+  </si>
+  <si>
+    <t>=+SUMIF(Bang_TSCD!$B$16:$B$5000,AC210,Bang_TSCD!$S$16:$S$5000)</t>
+  </si>
+  <si>
+    <t>VA26093001_16</t>
+  </si>
+  <si>
+    <t>K562</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(K559,Bang_CDSPSNT,4,0)/1000</t>
+  </si>
+  <si>
+    <t>TM muc 27: so du dau nam truoc lay tu CDSPS nam truoc</t>
+  </si>
+  <si>
+    <t>VA26093001_17</t>
+  </si>
+  <si>
+    <t>N562</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(N559,Bang_CDSPSNT,4,0)/1000-VLOOKUP(N559,Bang_CDSPSNT,3,0)/1000</t>
+  </si>
+  <si>
+    <t>VA26093001_18</t>
+  </si>
+  <si>
+    <t>Q562</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(Q559,Bang_CDSPSNT,4,0)/1000</t>
+  </si>
+  <si>
+    <t>VA26093001_19</t>
+  </si>
+  <si>
+    <t>T562</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(T559,Bang_CDSPSNT,4,0)/1000</t>
+  </si>
+  <si>
+    <t>VA26093001_20</t>
+  </si>
+  <si>
+    <t>W562</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(W559,Bang_CDSPSNT,4,0)/1000-VLOOKUP(W559,Bang_CDSPSNT,3,0)/1000</t>
+  </si>
+  <si>
+    <t>VA26093001_21</t>
+  </si>
+  <si>
+    <t>Z562</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(Z559,Bang_CDSPSNT,4,0)/1000-VLOOKUP(Z559,Bang_CDSPSNT,3,0)/1000</t>
+  </si>
+  <si>
+    <t>VA26093001_22</t>
+  </si>
+  <si>
+    <t>AC562</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(AC559,Bang_CDSPSNT,4,0)/1000-VLOOKUP(AC559,Bang_CDSPSNT,3,0)/1000</t>
+  </si>
+  <si>
+    <t>VA26093001_23</t>
+  </si>
+  <si>
+    <t>AF562</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(AF559,Bang_CDSPSNT,4,0)/1000</t>
+  </si>
+  <si>
+    <t>VA26093001_24</t>
+  </si>
+  <si>
+    <t>K563</t>
+  </si>
+  <si>
+    <t>=+VLOOKUP(K559,Bang_CDSPSNT,6,0)/1000</t>
+  </si>
+  <si>
+    <t>TM muc 27: tang von trong nam truoc</t>
+  </si>
+  <si>
+    <t>VA26093001_25</t>
+  </si>
+  <si>
+    <t>AC564</t>
+  </si>
+  <si>
+    <t>=+MAX(VLOOKUP(AC559,Bang_CDSPSNT,6,0)-VLOOKUP(AC559,Bang_CDSPSNT,5,0),0)/1000</t>
+  </si>
+  <si>
+    <t>TM muc 27: lai trong nam truoc</t>
+  </si>
+  <si>
+    <t>VA26093001_26</t>
+  </si>
+  <si>
+    <t>AC567</t>
+  </si>
+  <si>
+    <t>=+MAX(VLOOKUP(AC559,Bang_CDSPSNT,5,0)-VLOOKUP(AC559,Bang_CDSPSNT,6,0),0)/1000</t>
+  </si>
+  <si>
+    <t>TM muc 27: lo trong nam truoc</t>
+  </si>
+  <si>
+    <t>VA26093001_27</t>
+  </si>
+  <si>
+    <t>AL784</t>
+  </si>
+  <si>
+    <t>=IF(SUM(Y784:AK784)&gt;1,1,0)</t>
+  </si>
+  <si>
+    <t>TM: an/hien dong ghi chu (*) theo so lieu</t>
+  </si>
 </sst>
 </file>
 
@@ -812,7 +1087,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -925,6 +1200,7 @@
     <xf numFmtId="49" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1482,361 +1758,793 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="A9" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E9" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="I9" s="2"/>
       <c r="K9" s="39" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="A10" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E10" s="50" t="s">
+        <v>144</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="K10" s="39" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E11" s="50" t="s">
+        <v>147</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="I11" s="2"/>
       <c r="K11" s="39" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E12" s="50" t="s">
+        <v>150</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="I12" s="2"/>
       <c r="K12" s="39" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E13" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="I13" s="2"/>
       <c r="K13" s="39" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E14" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>157</v>
+      </c>
       <c r="I14" s="2"/>
       <c r="K14" s="39" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>160</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>157</v>
+      </c>
       <c r="I15" s="2"/>
       <c r="K15" s="39" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="A16" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E16" s="50" t="s">
+        <v>163</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>157</v>
+      </c>
       <c r="I16" s="2"/>
       <c r="K16" s="39"/>
     </row>
     <row r="17" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
+      <c r="A17" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E17" s="50" t="s">
+        <v>166</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>157</v>
+      </c>
       <c r="I17" s="2"/>
       <c r="K17" s="39" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
+      <c r="A18" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E18" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>157</v>
+      </c>
       <c r="I18" s="2"/>
       <c r="K18" s="39" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
+      <c r="A19" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>172</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>173</v>
+      </c>
       <c r="I19" s="2"/>
       <c r="K19" s="39" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
+      <c r="A20" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E20" s="50" t="s">
+        <v>176</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>173</v>
+      </c>
       <c r="I20" s="2"/>
       <c r="K20" s="39" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
+      <c r="A21" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>179</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>173</v>
+      </c>
       <c r="I21" s="2"/>
       <c r="K21" s="39"/>
     </row>
     <row r="22" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
+      <c r="A22" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="E22" s="50" t="s">
+        <v>182</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>173</v>
+      </c>
       <c r="I22" s="2"/>
       <c r="K22" s="39" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
+      <c r="A23" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E23" s="50" t="s">
+        <v>185</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>173</v>
+      </c>
       <c r="I23" s="2"/>
       <c r="K23" s="39" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
+      <c r="A24" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E24" s="50" t="s">
+        <v>188</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="I24" s="2"/>
       <c r="K24" s="39" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
+      <c r="A25" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>192</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="I25" s="2"/>
       <c r="K25" s="39" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
+      <c r="A26" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E26" s="50" t="s">
+        <v>195</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="I26" s="2"/>
       <c r="K26" s="39"/>
     </row>
     <row r="27" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
+      <c r="A27" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E27" s="50" t="s">
+        <v>198</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="I27" s="2"/>
       <c r="K27" s="39" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
+      <c r="A28" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E28" s="50" t="s">
+        <v>201</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="I28" s="2"/>
       <c r="K28" s="39"/>
     </row>
     <row r="29" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
+      <c r="A29" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E29" s="50" t="s">
+        <v>204</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="I29" s="2"/>
       <c r="K29" s="39" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
+      <c r="A30" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E30" s="50" t="s">
+        <v>207</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="I30" s="2"/>
       <c r="K30" s="39" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
+      <c r="A31" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E31" s="50" t="s">
+        <v>210</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="I31" s="2"/>
       <c r="K31" s="39" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
+      <c r="A32" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E32" s="50" t="s">
+        <v>213</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>214</v>
+      </c>
       <c r="I32" s="2"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
+      <c r="A33" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E33" s="50" t="s">
+        <v>217</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>218</v>
+      </c>
       <c r="I33" s="2"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
+      <c r="A34" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="E34" s="50" t="s">
+        <v>221</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>222</v>
+      </c>
       <c r="I34" s="2"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
+      <c r="A35" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E35" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>226</v>
+      </c>
       <c r="I35" s="2"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
phat hanh 26101101 (TT99 + LND + TT58): Fix lay du lieu File cu; kiem tra du lieu bang luong - cot Thang tinh PC kiem theo cap, khong lech khi them/bot cot phu cap (mau bieu schema 11)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MauBieu.xlsx
+++ b/MauBieu.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\AppData\Local\Temp\gpacc-dist-pub\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\AppData\Local\Temp\gpacc-dist-pub3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F468F3-F21E-45CE-B060-9BA8811D8CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD41150-E392-421B-B5AC-E7C366FB9E74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{65DAC49F-DB37-4ACF-9950-1AF1DBA8E511}"/>
   </bookViews>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="340">
   <si>
     <t>NK_Mua</t>
   </si>
@@ -976,6 +976,129 @@
   </si>
   <si>
     <t>LT cot Thang: BatBuoc 2 = chi bat buoc khi dong co dinh khoan (dong khong dinh khoan -&gt; khong bao loi)</t>
+  </si>
+  <si>
+    <t>VA26101101_01</t>
+  </si>
+  <si>
+    <t>B62</t>
+  </si>
+  <si>
+    <t>TTNV_PC</t>
+  </si>
+  <si>
+    <t>TTNV Phu cap: neo TTNV_PC, lap moi cot toi truoc TTNV_KTX (khach them/bot loai phu cap khong lech cot)</t>
+  </si>
+  <si>
+    <t>VA26101101_02</t>
+  </si>
+  <si>
+    <t>C62</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>VA26101101_03</t>
+  </si>
+  <si>
+    <t>F62</t>
+  </si>
+  <si>
+    <t>Phụ cấp</t>
+  </si>
+  <si>
+    <t>VA26101101_04</t>
+  </si>
+  <si>
+    <t>H62</t>
+  </si>
+  <si>
+    <t>LAP:1:TTNV_KTX</t>
+  </si>
+  <si>
+    <t>VA26101101_05</t>
+  </si>
+  <si>
+    <t>B63</t>
+  </si>
+  <si>
+    <t>TTNV_KTX</t>
+  </si>
+  <si>
+    <t>TTNV Phu cap khong thuong xuyen (tien): neo TTNV_KTX, lap moi 2 cot toi truoc TTNV_GC</t>
+  </si>
+  <si>
+    <t>VA26101101_06</t>
+  </si>
+  <si>
+    <t>C63</t>
+  </si>
+  <si>
+    <t>VA26101101_07</t>
+  </si>
+  <si>
+    <t>F63</t>
+  </si>
+  <si>
+    <t>Phụ cấp không thường xuyên</t>
+  </si>
+  <si>
+    <t>VA26101101_08</t>
+  </si>
+  <si>
+    <t>H63</t>
+  </si>
+  <si>
+    <t>LAP:2:TTNV_GC</t>
+  </si>
+  <si>
+    <t>VA26101101_09</t>
+  </si>
+  <si>
+    <t>B64</t>
+  </si>
+  <si>
+    <t>TTNV Thang tinh PC: neo TTNV_KTX cot 2, lap moi 2 cot toi truoc TTNV_GC (truoc day kiem nham cot tien)</t>
+  </si>
+  <si>
+    <t>VA26101101_10</t>
+  </si>
+  <si>
+    <t>C64</t>
+  </si>
+  <si>
+    <t>VA26101101_11</t>
+  </si>
+  <si>
+    <t>D64</t>
+  </si>
+  <si>
+    <t>THANG</t>
+  </si>
+  <si>
+    <t>VA26101101_12</t>
+  </si>
+  <si>
+    <t>F64</t>
+  </si>
+  <si>
+    <t>Tháng tính PC</t>
+  </si>
+  <si>
+    <t>VA26101101_13</t>
+  </si>
+  <si>
+    <t>H64</t>
+  </si>
+  <si>
+    <t>VA26101101_14</t>
+  </si>
+  <si>
+    <t>A65:H68</t>
+  </si>
+  <si>
+    <t>Bo 4 dong TTNV cu (PC nha o/khac/khong thuong xuyen/thang) - da gop vao 3 dong LAP o tren</t>
   </si>
 </sst>
 </file>
@@ -3177,157 +3300,351 @@
       <c r="I54" s="2"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
+      <c r="A55" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>301</v>
+      </c>
       <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
+      <c r="G55" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>302</v>
+      </c>
       <c r="I55" s="2"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
+      <c r="A56" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>305</v>
+      </c>
       <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
-      <c r="H56" s="2"/>
+      <c r="G56" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>302</v>
+      </c>
       <c r="I56" s="2"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
+      <c r="A57" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>308</v>
+      </c>
       <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
+      <c r="G57" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>302</v>
+      </c>
       <c r="I57" s="2"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
+      <c r="A58" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>311</v>
+      </c>
       <c r="F58" s="2"/>
-      <c r="G58" s="2"/>
-      <c r="H58" s="2"/>
+      <c r="G58" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>302</v>
+      </c>
       <c r="I58" s="2"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
+      <c r="A59" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>314</v>
+      </c>
       <c r="F59" s="2"/>
-      <c r="G59" s="2"/>
-      <c r="H59" s="2"/>
+      <c r="G59" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>315</v>
+      </c>
       <c r="I59" s="2"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
+      <c r="A60" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>305</v>
+      </c>
       <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="2"/>
+      <c r="G60" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>315</v>
+      </c>
       <c r="I60" s="2"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
+      <c r="A61" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>320</v>
+      </c>
       <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
-      <c r="H61" s="2"/>
+      <c r="G61" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>315</v>
+      </c>
       <c r="I61" s="2"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
+      <c r="A62" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>323</v>
+      </c>
       <c r="F62" s="2"/>
-      <c r="G62" s="2"/>
-      <c r="H62" s="2"/>
+      <c r="G62" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>315</v>
+      </c>
       <c r="I62" s="2"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
+      <c r="A63" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>314</v>
+      </c>
       <c r="F63" s="2"/>
-      <c r="G63" s="2"/>
-      <c r="H63" s="2"/>
+      <c r="G63" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="I63" s="2"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
+      <c r="A64" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>230</v>
+      </c>
       <c r="F64" s="2"/>
-      <c r="G64" s="2"/>
-      <c r="H64" s="2"/>
+      <c r="G64" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="I64" s="2"/>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
+      <c r="A65" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>331</v>
+      </c>
       <c r="F65" s="2"/>
-      <c r="G65" s="2"/>
-      <c r="H65" s="2"/>
+      <c r="G65" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="I65" s="2"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
+      <c r="A66" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>334</v>
+      </c>
       <c r="F66" s="2"/>
-      <c r="G66" s="2"/>
-      <c r="H66" s="2"/>
+      <c r="G66" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="I66" s="2"/>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
+      <c r="A67" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>323</v>
+      </c>
       <c r="F67" s="2"/>
-      <c r="G67" s="2"/>
-      <c r="H67" s="2"/>
+      <c r="G67" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="I67" s="2"/>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A68" s="2"/>
-      <c r="B68" s="2"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
+      <c r="A68" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>338</v>
+      </c>
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
-      <c r="G68" s="2"/>
-      <c r="H68" s="2"/>
+      <c r="G68" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>339</v>
+      </c>
       <c r="I68" s="2"/>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
phat hanh 26101301 (TT99 + LND + TT58): to khai GTGT xet hoa don mua vao theo thang ghi so; ket chuyen to khai tu ghi [37]/[38] khi bat hoa don muon + nut Ket Chuyen tren so DC_3738; mau bieu schema 12
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MauBieu.xlsx
+++ b/MauBieu.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\AppData\Local\Temp\gpacc-dist-pub3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\AppData\Local\Temp\gpacc-dist-pub5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD41150-E392-421B-B5AC-E7C366FB9E74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A876762-9A43-49B7-B4D9-B9B166F8CD58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{65DAC49F-DB37-4ACF-9950-1AF1DBA8E511}"/>
   </bookViews>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="351">
   <si>
     <t>NK_Mua</t>
   </si>
@@ -1099,6 +1099,39 @@
   </si>
   <si>
     <t>Bo 4 dong TTNV cu (PC nha o/khac/khong thuong xuyen/thang) - da gop vao 3 dong LAP o tren</t>
+  </si>
+  <si>
+    <t>VA26101301_01</t>
+  </si>
+  <si>
+    <t>KB_BoChanNKC</t>
+  </si>
+  <si>
+    <t>=TTDN!$J$42</t>
+  </si>
+  <si>
+    <t>Cong tac an (chi bao rieng khach can): 1 = ket chuyen NKC lech doi chieu PB-KH van giu so NKC/CDSPS, chi bao; 0 = chan nhu cu</t>
+  </si>
+  <si>
+    <t>VA26101301_02</t>
+  </si>
+  <si>
+    <t>J42</t>
+  </si>
+  <si>
+    <t>Cong tac KB_BoChanNKC mac dinh 0 - chi dat khi o con trong</t>
+  </si>
+  <si>
+    <t>VA26101301_03</t>
+  </si>
+  <si>
+    <t>Cong tac KB_BoChanNKC: o khong nhan, chu xam nho</t>
+  </si>
+  <si>
+    <t>VA26101301_04</t>
+  </si>
+  <si>
+    <t>Cong tac KB_BoChanNKC chi nhan 0 hoac 1</t>
   </si>
 </sst>
 </file>
@@ -3648,47 +3681,103 @@
       <c r="I68" s="2"/>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
+      <c r="A69" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="E69" s="40" t="s">
+        <v>342</v>
+      </c>
       <c r="F69" s="2"/>
-      <c r="G69" s="2"/>
-      <c r="H69" s="2"/>
+      <c r="G69" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>343</v>
+      </c>
       <c r="I69" s="2"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
+      <c r="A70" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>273</v>
+      </c>
       <c r="F70" s="2"/>
-      <c r="G70" s="2"/>
-      <c r="H70" s="2"/>
+      <c r="G70" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>346</v>
+      </c>
       <c r="I70" s="2"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
+      <c r="A71" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>345</v>
+      </c>
       <c r="E71" s="2"/>
-      <c r="F71" s="2"/>
-      <c r="G71" s="2"/>
-      <c r="H71" s="2"/>
+      <c r="F71" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="I71" s="2"/>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A72" s="2"/>
-      <c r="B72" s="2"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="E72" s="2"/>
+      <c r="A72" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>280</v>
+      </c>
       <c r="F72" s="2"/>
-      <c r="G72" s="2"/>
-      <c r="H72" s="2"/>
+      <c r="G72" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>350</v>
+      </c>
       <c r="I72" s="2"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
phat hanh 26101701 (TT99 + LND + TT58): Keo DL tu GPAcc PRO (cong 8831, hoi khi nhieu phan mem); to khai TNCN 05QTT tach cu tru/khong cu tru PL_052, Khong phat sinh khong tinh lao dong, HDLD + CTV dem 1 nguoi, [21] so ca nhan giam tru; 05KK dem HDLD moi dong
</commit_message>
<xml_diff>
--- a/MauBieu.xlsx
+++ b/MauBieu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\AppData\Local\Temp\gpacc-dist-pub5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\AppData\Local\Temp\gpacc-dist-pub11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A876762-9A43-49B7-B4D9-B9B166F8CD58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34734242-9D75-4034-AB26-E4043CCC8907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{65DAC49F-DB37-4ACF-9950-1AF1DBA8E511}"/>
+    <workbookView xWindow="15310" yWindow="1520" windowWidth="19880" windowHeight="15370" xr2:uid="{65DAC49F-DB37-4ACF-9950-1AF1DBA8E511}"/>
   </bookViews>
   <sheets>
     <sheet name="VA_BOCUC" sheetId="4" r:id="rId1"/>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="396">
   <si>
     <t>NK_Mua</t>
   </si>
@@ -1132,6 +1132,141 @@
   </si>
   <si>
     <t>Cong tac KB_BoChanNKC chi nhan 0 hoac 1</t>
+  </si>
+  <si>
+    <t>VA26101701_01</t>
+  </si>
+  <si>
+    <t>05QTT</t>
+  </si>
+  <si>
+    <t>I26</t>
+  </si>
+  <si>
+    <t>=COUNT(INDEX(PL_051!$B:$B,ROW(PL051_A)+1):INDEX(PL_051!$B:$B,ROW(PL051_TC)-1))+SUMPRODUCT(ISNUMBER(INDEX(PL_052!$B:$B,ROW(PL052_A)+1):INDEX(PL_052!$B:$B,ROW(PL052_TC)-1))*(COUNTIFS(INDEX(PL_051!$C:$C,ROW(PL051_A)+1):INDEX(PL_051!$C:$C,ROW(PL051_TC)-1),INDEX(PL_052!$C:$C,ROW(PL052_A)+1):INDEX(PL_052!$C:$C,ROW(PL052_TC)-1)&amp;"",INDEX(PL_051!$D:$D,ROW(PL051_A)+1):INDEX(PL_051!$D:$D,ROW(PL051_TC)-1),INDEX(PL_052!$D:$D,ROW(PL052_A)+1):INDEX(PL_052!$D:$D,ROW(PL052_TC)-1)&amp;"",INDEX(PL_051!$E:$E,ROW(PL051_A)+1):INDEX(PL_051!$E:$E,ROW(PL051_TC)-1),INDEX(PL_052!$E:$E,ROW(PL052_A)+1):INDEX(PL_052!$E:$E,ROW(PL052_TC)-1)&amp;"")=0))</t>
+  </si>
+  <si>
+    <t>05QTT [15]: dem theo STT (bo chu Khong phat sinh); nguoi vua HDLD vua CTV dem 1 lan</t>
+  </si>
+  <si>
+    <t>VA26101701_02</t>
+  </si>
+  <si>
+    <t>I27</t>
+  </si>
+  <si>
+    <t>=COUNT(INDEX(PL_051!$B:$B,ROW(PL051_A)+1):INDEX(PL_051!$B:$B,ROW(PL051_TC)-1))</t>
+  </si>
+  <si>
+    <t>05QTT [16]: dem theo STT (bo chu Khong phat sinh)</t>
+  </si>
+  <si>
+    <t>VA26101701_03</t>
+  </si>
+  <si>
+    <t>I29</t>
+  </si>
+  <si>
+    <t>=COUNTIF(INDEX(PL_051!$P:$P,ROW(PL051_A)+1):INDEX(PL_051!$P:$P,ROW(PL051_TC)-1),"&gt;0")+SUMPRODUCT(ISNUMBER(INDEX(PL_052!$B:$B,ROW(PL052_A)+1):INDEX(PL_052!$B:$B,ROW(PL052_TC)-1))*(INDEX(PL_052!$F:$F,ROW(PL052_A)+1):INDEX(PL_052!$F:$F,ROW(PL052_TC)-1)&lt;&gt;"x")*(INDEX(PL_052!$K:$K,ROW(PL052_A)+1):INDEX(PL_052!$K:$K,ROW(PL052_TC)-1)&gt;0)*(COUNTIFS(INDEX(PL_051!$C:$C,ROW(PL051_A)+1):INDEX(PL_051!$C:$C,ROW(PL051_TC)-1),INDEX(PL_052!$C:$C,ROW(PL052_A)+1):INDEX(PL_052!$C:$C,ROW(PL052_TC)-1)&amp;"",INDEX(PL_051!$D:$D,ROW(PL051_A)+1):INDEX(PL_051!$D:$D,ROW(PL051_TC)-1),INDEX(PL_052!$D:$D,ROW(PL052_A)+1):INDEX(PL_052!$D:$D,ROW(PL052_TC)-1)&amp;"",INDEX(PL_051!$E:$E,ROW(PL051_A)+1):INDEX(PL_051!$E:$E,ROW(PL051_TC)-1),INDEX(PL_052!$E:$E,ROW(PL052_A)+1):INDEX(PL_052!$E:$E,ROW(PL052_TC)-1)&amp;"",INDEX(PL_051!$P:$P,ROW(PL051_A)+1):INDEX(PL_051!$P:$P,ROW(PL051_TC)-1),"&gt;0")=0))</t>
+  </si>
+  <si>
+    <t>05QTT [18]: + ca nhan CU TRU cua PL_052 (CTV 10%) da khau tru; nguoi o ca 2 bang dem 1 lan</t>
+  </si>
+  <si>
+    <t>VA26101701_04</t>
+  </si>
+  <si>
+    <t>I30</t>
+  </si>
+  <si>
+    <t>=COUNTIFS(INDEX(PL_052!$K:$K,ROW(PL052_A)+1):INDEX(PL_052!$K:$K,ROW(PL052_TC)-1),"&gt;0",INDEX(PL_052!$F:$F,ROW(PL052_A)+1):INDEX(PL_052!$F:$F,ROW(PL052_TC)-1),"x")</t>
+  </si>
+  <si>
+    <t>05QTT [19]: chi ca nhan KHONG cu tru (PL_052 cot F = x)</t>
+  </si>
+  <si>
+    <t>VA26101701_05</t>
+  </si>
+  <si>
+    <t>I32</t>
+  </si>
+  <si>
+    <t>=COUNTIF(INDEX(PL_051!$K:$K,ROW(PL051_A)+1):INDEX(PL_051!$K:$K,ROW(PL051_TC)-1),"&gt;0")</t>
+  </si>
+  <si>
+    <t>05QTT [21]: so ca nhan co giam tru gia canh (truoc cong so nguoi phu thuoc)</t>
+  </si>
+  <si>
+    <t>VA26101701_06</t>
+  </si>
+  <si>
+    <t>I34</t>
+  </si>
+  <si>
+    <t>=SUM(INDEX(PL_051!$G:$G,ROW(PL051_A)+1):INDEX(PL_051!$G:$G,ROW(PL051_TC)-1))+SUMIFS(INDEX(PL_052!$G:$G,ROW(PL052_A)+1):INDEX(PL_052!$G:$G,ROW(PL052_TC)-1),INDEX(PL_052!$F:$F,ROW(PL052_A)+1):INDEX(PL_052!$F:$F,ROW(PL052_TC)-1),"&lt;&gt;x")</t>
+  </si>
+  <si>
+    <t>05QTT [23]: + thu nhap ca nhan cu tru cua PL_052</t>
+  </si>
+  <si>
+    <t>VA26101701_07</t>
+  </si>
+  <si>
+    <t>I35</t>
+  </si>
+  <si>
+    <t>=SUMIFS(INDEX(PL_052!$G:$G,ROW(PL052_A)+1):INDEX(PL_052!$G:$G,ROW(PL052_TC)-1),INDEX(PL_052!$F:$F,ROW(PL052_A)+1):INDEX(PL_052!$F:$F,ROW(PL052_TC)-1),"x")</t>
+  </si>
+  <si>
+    <t>05QTT [24]: chi ca nhan khong cu tru</t>
+  </si>
+  <si>
+    <t>VA26101701_08</t>
+  </si>
+  <si>
+    <t>I42</t>
+  </si>
+  <si>
+    <t>=SUMIFS(INDEX(PL_051!$G:$G,ROW(PL051_A)+1):INDEX(PL_051!$G:$G,ROW(PL051_TC)-1),INDEX(PL_051!$P:$P,ROW(PL051_A)+1):INDEX(PL_051!$P:$P,ROW(PL051_TC)-1),"&gt;0")+SUMIFS(INDEX(PL_052!$G:$G,ROW(PL052_A)+1):INDEX(PL_052!$G:$G,ROW(PL052_TC)-1),INDEX(PL_052!$K:$K,ROW(PL052_A)+1):INDEX(PL_052!$K:$K,ROW(PL052_TC)-1),"&gt;0",INDEX(PL_052!$F:$F,ROW(PL052_A)+1):INDEX(PL_052!$F:$F,ROW(PL052_TC)-1),"&lt;&gt;x")</t>
+  </si>
+  <si>
+    <t>05QTT [31]: + ca nhan cu tru cua PL_052 thuoc dien khau tru</t>
+  </si>
+  <si>
+    <t>VA26101701_09</t>
+  </si>
+  <si>
+    <t>I43</t>
+  </si>
+  <si>
+    <t>=SUMIFS(INDEX(PL_052!$G:$G,ROW(PL052_A)+1):INDEX(PL_052!$G:$G,ROW(PL052_TC)-1),INDEX(PL_052!$K:$K,ROW(PL052_A)+1):INDEX(PL_052!$K:$K,ROW(PL052_TC)-1),"&gt;0",INDEX(PL_052!$F:$F,ROW(PL052_A)+1):INDEX(PL_052!$F:$F,ROW(PL052_TC)-1),"x")</t>
+  </si>
+  <si>
+    <t>05QTT [32]: chi ca nhan khong cu tru</t>
+  </si>
+  <si>
+    <t>VA26101701_10</t>
+  </si>
+  <si>
+    <t>I45</t>
+  </si>
+  <si>
+    <t>=SUM(INDEX(PL_051!$P:$P,ROW(PL051_A)+1):INDEX(PL_051!$P:$P,ROW(PL051_TC)-1))+SUMIFS(INDEX(PL_052!$K:$K,ROW(PL052_A)+1):INDEX(PL_052!$K:$K,ROW(PL052_TC)-1),INDEX(PL_052!$F:$F,ROW(PL052_A)+1):INDEX(PL_052!$F:$F,ROW(PL052_TC)-1),"&lt;&gt;x")</t>
+  </si>
+  <si>
+    <t>05QTT [34]: + thue da khau tru cua ca nhan cu tru PL_052</t>
+  </si>
+  <si>
+    <t>VA26101701_11</t>
+  </si>
+  <si>
+    <t>I46</t>
+  </si>
+  <si>
+    <t>=SUMIFS(INDEX(PL_052!$K:$K,ROW(PL052_A)+1):INDEX(PL_052!$K:$K,ROW(PL052_TC)-1),INDEX(PL_052!$F:$F,ROW(PL052_A)+1):INDEX(PL_052!$F:$F,ROW(PL052_TC)-1),"x")</t>
+  </si>
+  <si>
+    <t>05QTT [35]: chi ca nhan khong cu tru</t>
   </si>
 </sst>
 </file>
@@ -3781,124 +3916,278 @@
       <c r="I72" s="2"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A73" s="2"/>
-      <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
+      <c r="A73" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="E73" s="40" t="s">
+        <v>354</v>
+      </c>
       <c r="F73" s="2"/>
-      <c r="G73" s="2"/>
-      <c r="H73" s="2"/>
+      <c r="G73" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>355</v>
+      </c>
       <c r="I73" s="2"/>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A74" s="2"/>
-      <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
+      <c r="A74" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="E74" s="40" t="s">
+        <v>358</v>
+      </c>
       <c r="F74" s="2"/>
-      <c r="G74" s="2"/>
-      <c r="H74" s="2"/>
+      <c r="G74" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>359</v>
+      </c>
       <c r="I74" s="2"/>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A75" s="2"/>
-      <c r="B75" s="2"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
+      <c r="A75" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="E75" s="40" t="s">
+        <v>362</v>
+      </c>
       <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
-      <c r="H75" s="2"/>
+      <c r="G75" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>363</v>
+      </c>
       <c r="I75" s="2"/>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
+      <c r="A76" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E76" s="40" t="s">
+        <v>366</v>
+      </c>
       <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
-      <c r="H76" s="2"/>
+      <c r="G76" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>367</v>
+      </c>
       <c r="I76" s="2"/>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A77" s="2"/>
-      <c r="B77" s="2"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
+      <c r="A77" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E77" s="40" t="s">
+        <v>370</v>
+      </c>
       <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
-      <c r="H77" s="2"/>
+      <c r="G77" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H77" s="2" t="s">
+        <v>371</v>
+      </c>
       <c r="I77" s="2"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A78" s="2"/>
-      <c r="B78" s="2"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
+      <c r="A78" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="E78" s="40" t="s">
+        <v>374</v>
+      </c>
       <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
-      <c r="H78" s="2"/>
+      <c r="G78" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>375</v>
+      </c>
       <c r="I78" s="2"/>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A79" s="2"/>
-      <c r="B79" s="2"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
+      <c r="A79" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="E79" s="40" t="s">
+        <v>378</v>
+      </c>
       <c r="F79" s="2"/>
-      <c r="G79" s="2"/>
-      <c r="H79" s="2"/>
+      <c r="G79" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>379</v>
+      </c>
       <c r="I79" s="2"/>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A80" s="2"/>
-      <c r="B80" s="2"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
+      <c r="A80" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="E80" s="40" t="s">
+        <v>382</v>
+      </c>
       <c r="F80" s="2"/>
-      <c r="G80" s="2"/>
-      <c r="H80" s="2"/>
+      <c r="G80" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>383</v>
+      </c>
       <c r="I80" s="2"/>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A81" s="2"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
+      <c r="A81" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="E81" s="40" t="s">
+        <v>386</v>
+      </c>
       <c r="F81" s="2"/>
-      <c r="G81" s="2"/>
-      <c r="H81" s="2"/>
+      <c r="G81" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>387</v>
+      </c>
       <c r="I81" s="2"/>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
+      <c r="A82" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="E82" s="40" t="s">
+        <v>390</v>
+      </c>
       <c r="F82" s="2"/>
-      <c r="G82" s="2"/>
-      <c r="H82" s="2"/>
+      <c r="G82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>391</v>
+      </c>
       <c r="I82" s="2"/>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A83" s="2"/>
-      <c r="B83" s="2"/>
-      <c r="C83" s="2"/>
-      <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
+      <c r="A83" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E83" s="40" t="s">
+        <v>394</v>
+      </c>
       <c r="F83" s="2"/>
-      <c r="G83" s="2"/>
-      <c r="H83" s="2"/>
+      <c r="G83" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>395</v>
+      </c>
       <c r="I83" s="2"/>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>